<commit_message>
Adding offshore slope to templates. Adding Berm to floodwalls.
</commit_message>
<xml_diff>
--- a/SS_levee_input.xlsx
+++ b/SS_levee_input.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\0_StormSim_Task\StormSim-Library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A801A25B-117A-42F4-B15E-4FF434AF2DB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2D99B5D-02F5-456C-8C9C-ADCC797A59C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="23955" windowHeight="20985" xr2:uid="{E6B7D8F3-466A-4168-A43B-4ED2ECFB7BAF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{E6B7D8F3-466A-4168-A43B-4ED2ECFB7BAF}"/>
   </bookViews>
   <sheets>
     <sheet name="Levee" sheetId="1" r:id="rId1"/>
@@ -41,12 +41,6 @@
     <t>NA</t>
   </si>
   <si>
-    <t>Bottom Slope To Use For Damaging Dpeths (tanb)</t>
-  </si>
-  <si>
-    <t>compute_damaging_depth_slope</t>
-  </si>
-  <si>
     <t>Shielding Parameter To Use For Damaging Depths</t>
   </si>
   <si>
@@ -426,6 +420,12 @@
   </si>
   <si>
     <t>..\CHS_Dependencies</t>
+  </si>
+  <si>
+    <t>offshore_slope</t>
+  </si>
+  <si>
+    <t>Offshore slope (cota)</t>
   </si>
 </sst>
 </file>
@@ -468,7 +468,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -496,12 +496,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -536,7 +530,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -693,11 +687,42 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -734,26 +759,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -761,7 +766,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -776,21 +781,21 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -802,8 +807,41 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1133,96 +1171,96 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
-        <v>124</v>
-      </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="F1" s="45" t="s">
-        <v>90</v>
-      </c>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40" t="s">
-        <v>89</v>
-      </c>
-      <c r="I1" s="40" t="s">
-        <v>89</v>
+      <c r="A1" s="40" t="s">
+        <v>122</v>
+      </c>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="F1" s="39" t="s">
+        <v>88</v>
+      </c>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34" t="s">
+        <v>87</v>
+      </c>
+      <c r="I1" s="34" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C2" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>15</v>
-      </c>
       <c r="H2" s="6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="22" t="s">
-        <v>123</v>
-      </c>
-      <c r="B3" s="29" t="s">
-        <v>122</v>
-      </c>
-      <c r="C3" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="D3" s="27" t="s">
+      <c r="A3" s="16" t="s">
         <v>121</v>
       </c>
-      <c r="F3" s="44" t="s">
-        <v>84</v>
-      </c>
-      <c r="G3" s="43" t="s">
-        <v>83</v>
-      </c>
-      <c r="H3" s="42" t="s">
-        <v>0</v>
-      </c>
-      <c r="I3" s="41">
+      <c r="B3" s="23" t="s">
+        <v>120</v>
+      </c>
+      <c r="C3" s="22" t="s">
+        <v>0</v>
+      </c>
+      <c r="D3" s="21" t="s">
+        <v>119</v>
+      </c>
+      <c r="F3" s="38" t="s">
+        <v>82</v>
+      </c>
+      <c r="G3" s="37" t="s">
+        <v>81</v>
+      </c>
+      <c r="H3" s="36" t="s">
+        <v>0</v>
+      </c>
+      <c r="I3" s="35">
         <v>1000</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="I4" s="2">
         <v>50</v>
@@ -1230,112 +1268,112 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>0</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40"/>
-      <c r="H5" s="40"/>
-      <c r="I5" s="40"/>
+        <v>113</v>
+      </c>
+      <c r="F5" s="34"/>
+      <c r="G5" s="34"/>
+      <c r="H5" s="34"/>
+      <c r="I5" s="34"/>
     </row>
     <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>0</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="F6" s="39" t="s">
-        <v>73</v>
-      </c>
-      <c r="G6" s="34"/>
-      <c r="H6" s="34"/>
-      <c r="I6" s="34"/>
+        <v>110</v>
+      </c>
+      <c r="F6" s="33" t="s">
+        <v>71</v>
+      </c>
+      <c r="G6" s="28"/>
+      <c r="H6" s="28"/>
+      <c r="I6" s="28"/>
     </row>
     <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="D7" s="2" t="s">
         <v>109</v>
       </c>
+      <c r="B7" s="50" t="s">
+        <v>108</v>
+      </c>
+      <c r="C7" s="51" t="s">
+        <v>0</v>
+      </c>
+      <c r="D7" s="52" t="s">
+        <v>107</v>
+      </c>
       <c r="F7" s="7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="D8" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="F8" s="22" t="s">
-        <v>70</v>
-      </c>
-      <c r="G8" s="29" t="s">
-        <v>69</v>
-      </c>
-      <c r="H8" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="I8" s="27">
+      <c r="B8" s="50" t="s">
+        <v>105</v>
+      </c>
+      <c r="C8" s="51" t="s">
+        <v>0</v>
+      </c>
+      <c r="D8" s="52" t="s">
+        <v>104</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="G8" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="H8" s="22" t="s">
+        <v>0</v>
+      </c>
+      <c r="I8" s="21">
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="D9" s="2">
+        <v>103</v>
+      </c>
+      <c r="B9" s="50" t="s">
+        <v>102</v>
+      </c>
+      <c r="C9" s="51" t="s">
+        <v>0</v>
+      </c>
+      <c r="D9" s="52">
         <v>1</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>0</v>
@@ -1346,22 +1384,22 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="B10" s="18" t="s">
-        <v>102</v>
-      </c>
-      <c r="C10" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="D10" s="16">
+        <v>101</v>
+      </c>
+      <c r="B10" s="50" t="s">
+        <v>100</v>
+      </c>
+      <c r="C10" s="51" t="s">
+        <v>0</v>
+      </c>
+      <c r="D10" s="52">
         <v>1</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>0</v>
@@ -1372,100 +1410,100 @@
     </row>
     <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="D11" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="F11" s="24" t="s">
-        <v>59</v>
+      <c r="B11" s="50" t="s">
+        <v>98</v>
+      </c>
+      <c r="C11" s="51" t="s">
+        <v>0</v>
+      </c>
+      <c r="D11" s="52" t="s">
+        <v>97</v>
+      </c>
+      <c r="F11" s="18" t="s">
+        <v>57</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H11" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="I11" s="23">
+        <v>22</v>
+      </c>
+      <c r="I11" s="17">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D12" s="2">
+        <v>96</v>
+      </c>
+      <c r="B12" s="50" t="s">
+        <v>95</v>
+      </c>
+      <c r="C12" s="51" t="s">
+        <v>22</v>
+      </c>
+      <c r="D12" s="52">
         <v>176.45</v>
       </c>
-      <c r="F12" s="34"/>
-      <c r="G12" s="34"/>
-      <c r="H12" s="34"/>
-      <c r="I12" s="34"/>
+      <c r="F12" s="28"/>
+      <c r="G12" s="28"/>
+      <c r="H12" s="28"/>
+      <c r="I12" s="28"/>
     </row>
     <row r="13" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="D13" s="2">
-        <v>0</v>
-      </c>
-      <c r="F13" s="33" t="s">
-        <v>54</v>
-      </c>
-      <c r="G13" s="32"/>
-      <c r="H13" s="32"/>
-      <c r="I13" s="32"/>
+        <v>94</v>
+      </c>
+      <c r="B13" s="50" t="s">
+        <v>93</v>
+      </c>
+      <c r="C13" s="51" t="s">
+        <v>0</v>
+      </c>
+      <c r="D13" s="52">
+        <v>0</v>
+      </c>
+      <c r="F13" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="G13" s="26"/>
+      <c r="H13" s="26"/>
+      <c r="I13" s="26"/>
     </row>
     <row r="14" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="D14" s="2">
+        <v>92</v>
+      </c>
+      <c r="B14" s="50" t="s">
+        <v>91</v>
+      </c>
+      <c r="C14" s="51" t="s">
+        <v>0</v>
+      </c>
+      <c r="D14" s="52">
         <v>1</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>0</v>
@@ -1473,25 +1511,25 @@
       <c r="D15" s="2">
         <v>0</v>
       </c>
-      <c r="F15" s="30" t="s">
-        <v>53</v>
-      </c>
-      <c r="G15" s="29" t="s">
-        <v>52</v>
-      </c>
-      <c r="H15" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="I15" s="27">
+      <c r="F15" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="G15" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="H15" s="22" t="s">
+        <v>0</v>
+      </c>
+      <c r="I15" s="21">
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>0</v>
@@ -1500,10 +1538,10 @@
         <v>1</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>0</v>
@@ -1514,10 +1552,10 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>0</v>
@@ -1526,10 +1564,10 @@
         <v>0</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="H17" s="3" t="s">
         <v>0</v>
@@ -1540,10 +1578,10 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>0</v>
@@ -1552,10 +1590,10 @@
         <v>0</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="H18" s="3" t="s">
         <v>0</v>
@@ -1566,22 +1604,22 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>0</v>
       </c>
       <c r="D19" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H19" s="3" t="s">
         <v>0</v>
@@ -1592,10 +1630,10 @@
     </row>
     <row r="20" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>0</v>
@@ -1603,207 +1641,207 @@
       <c r="D20" s="2">
         <v>1</v>
       </c>
-      <c r="F20" s="24" t="s">
-        <v>36</v>
+      <c r="F20" s="18" t="s">
+        <v>34</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H20" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="I20" s="23">
+      <c r="I20" s="17">
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="24" t="s">
-        <v>72</v>
+      <c r="A21" s="18" t="s">
+        <v>70</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="D21" s="23" t="s">
-        <v>44</v>
+      <c r="D21" s="17" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="38"/>
-      <c r="B22" s="37"/>
-      <c r="C22" s="36"/>
-      <c r="D22" s="36"/>
+      <c r="A22" s="32"/>
+      <c r="B22" s="31"/>
+      <c r="C22" s="30"/>
+      <c r="D22" s="30"/>
     </row>
     <row r="23" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="35" t="s">
-        <v>68</v>
-      </c>
-      <c r="B23" s="26"/>
-      <c r="C23" s="26"/>
-      <c r="D23" s="26"/>
+      <c r="A23" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="B23" s="20"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
     </row>
     <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="22" t="s">
-        <v>62</v>
-      </c>
-      <c r="B25" s="29" t="s">
-        <v>61</v>
-      </c>
-      <c r="C25" s="31" t="s">
+      <c r="A25" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="D25" s="27">
+      <c r="B25" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C25" s="25" t="s">
+        <v>58</v>
+      </c>
+      <c r="D25" s="21">
         <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="B26" s="29" t="s">
-        <v>56</v>
-      </c>
-      <c r="C26" s="31" t="s">
+      <c r="A26" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="D26" s="27">
+      <c r="B26" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="C26" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="D26" s="21">
         <v>2.46</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="22" t="s">
+      <c r="A27" s="16" t="s">
+        <v>125</v>
+      </c>
+      <c r="B27" s="23" t="s">
+        <v>126</v>
+      </c>
+      <c r="C27" s="25" t="s">
+        <v>0</v>
+      </c>
+      <c r="D27" s="21" t="s">
         <v>127</v>
-      </c>
-      <c r="B27" s="29" t="s">
-        <v>128</v>
-      </c>
-      <c r="C27" s="31" t="s">
-        <v>0</v>
-      </c>
-      <c r="D27" s="27" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>0</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>0</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="26"/>
-      <c r="B30" s="26"/>
-      <c r="C30" s="26"/>
-      <c r="D30" s="26"/>
+      <c r="A30" s="20"/>
+      <c r="B30" s="20"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="20"/>
     </row>
     <row r="31" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="B31" s="25"/>
-      <c r="C31" s="25"/>
-      <c r="D31" s="25"/>
+        <v>37</v>
+      </c>
+      <c r="B31" s="19"/>
+      <c r="C31" s="19"/>
+      <c r="D31" s="19"/>
     </row>
     <row r="32" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="22" t="s">
-        <v>34</v>
-      </c>
-      <c r="B33" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="C33" s="20" t="s">
-        <v>24</v>
-      </c>
-      <c r="D33" s="19">
+      <c r="A33" s="45" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33" s="46" t="s">
+        <v>31</v>
+      </c>
+      <c r="C33" s="47" t="s">
+        <v>22</v>
+      </c>
+      <c r="D33" s="48">
         <v>180.1</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B34" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="C34" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="D34" s="16">
+      <c r="A34" s="49" t="s">
+        <v>30</v>
+      </c>
+      <c r="B34" s="50" t="s">
+        <v>29</v>
+      </c>
+      <c r="C34" s="51" t="s">
+        <v>22</v>
+      </c>
+      <c r="D34" s="52">
         <v>0.3</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D35" s="2">
+      <c r="A35" s="49" t="s">
+        <v>28</v>
+      </c>
+      <c r="B35" s="50" t="s">
+        <v>27</v>
+      </c>
+      <c r="C35" s="51" t="s">
+        <v>22</v>
+      </c>
+      <c r="D35" s="52">
         <v>-1</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>0</v>
@@ -1814,10 +1852,10 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>0</v>
@@ -1826,102 +1864,103 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="15"/>
-      <c r="B38" s="15"/>
-      <c r="C38" s="15"/>
-      <c r="D38" s="15"/>
-    </row>
-    <row r="39" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="B39" s="9"/>
-      <c r="C39" s="9"/>
-      <c r="D39" s="9"/>
+    <row r="38" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="41" t="s">
+        <v>128</v>
+      </c>
+      <c r="B38" s="42" t="s">
+        <v>129</v>
+      </c>
+      <c r="C38" s="43" t="s">
+        <v>0</v>
+      </c>
+      <c r="D38" s="44">
+        <f>1/8</f>
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="15"/>
+      <c r="B39" s="15"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="15"/>
     </row>
     <row r="40" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="7" t="s">
+      <c r="A40" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="B40" s="9"/>
+      <c r="C40" s="9"/>
+      <c r="D40" s="9"/>
+    </row>
+    <row r="41" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D42" s="2">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B43" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="B40" s="6" t="s">
+      <c r="C43" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="D43" s="10">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="9"/>
+      <c r="B44" s="9"/>
+      <c r="C44" s="9"/>
+      <c r="D44" s="9"/>
+    </row>
+    <row r="45" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C40" s="6" t="s">
+      <c r="B45" s="1"/>
+      <c r="C45" s="1"/>
+      <c r="D45" s="1"/>
+    </row>
+    <row r="46" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D40" s="6" t="s">
+      <c r="B46" s="6" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C41" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D41" s="2">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="B42" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="C42" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="D42" s="10">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="9"/>
-      <c r="B43" s="9"/>
-      <c r="C43" s="9"/>
-      <c r="D43" s="9"/>
-    </row>
-    <row r="44" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B44" s="1"/>
-      <c r="C44" s="1"/>
-      <c r="D44" s="1"/>
-    </row>
-    <row r="45" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B45" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C45" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D45" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="5" t="s">
+      <c r="C46" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B46" s="4" t="s">
+      <c r="D46" s="6" t="s">
         <v>11</v>
-      </c>
-      <c r="C46" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="D46" s="2">
-        <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
@@ -1954,10 +1993,10 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
-        <v>125</v>
+        <v>6</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>126</v>
+        <v>5</v>
       </c>
       <c r="C49" s="3" t="s">
         <v>0</v>
@@ -1968,16 +2007,16 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
-        <v>6</v>
+        <v>123</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>5</v>
+        <v>124</v>
       </c>
       <c r="C50" s="3" t="s">
         <v>0</v>
       </c>
       <c r="D50" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -1991,7 +2030,7 @@
         <v>0</v>
       </c>
       <c r="D51" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -2005,7 +2044,7 @@
         <v>0</v>
       </c>
       <c r="D52" s="2">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -2021,7 +2060,7 @@
   <sheetProtection formatColumns="0" selectLockedCells="1"/>
   <protectedRanges>
     <protectedRange sqref="I15 I3:I4 I8:I11" name="Range1_1"/>
-    <protectedRange sqref="D41:D42" name="Range1_1_4"/>
+    <protectedRange sqref="D42:D43" name="Range1_1_4"/>
     <protectedRange sqref="D14 D16:D18 D9:D12 D6" name="Range1_1_1"/>
     <protectedRange sqref="D8 D15" name="Range1_1_1_1"/>
     <protectedRange sqref="D13" name="Range1_1_2"/>
@@ -2038,6 +2077,7 @@
     <protectedRange sqref="D29" name="Range1_1_2_1_1_1"/>
     <protectedRange sqref="D26:D27" name="Range1_1_5_2_1"/>
     <protectedRange sqref="D28" name="Range1_1_8_1_1_1"/>
+    <protectedRange sqref="D38" name="Range1_1_3_1_8_1"/>
   </protectedRanges>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>